<commit_message>
Milestone 4: Universal Indian listed-company discovery and financial intelligence engine
</commit_message>
<xml_diff>
--- a/data/company_intelligence/BHARATFORG/reports/bharat_forge_company_intelligence.xlsx
+++ b/data/company_intelligence/BHARATFORG/reports/bharat_forge_company_intelligence.xlsx
@@ -644,7 +644,7 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Capital Goods</t>
+          <t>Capital Goods &amp; Automotive</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>1961</t>
+          <t>1980</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
@@ -708,11 +708,7 @@
           <t>Registered Office</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Mundhwa, Pune Cantonment, Pune - 411036, Maharashtra, India</t>
-        </is>
-      </c>
+      <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Disclosed</t>
@@ -2117,7 +2113,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>835586603208afff9163fc3105d6a391c6a2c534623fe200233d87769ab3d321</t>
+          <t>7478a05ec6b106e73afa2202a98810527a911c6dfad3c69ecdc2709a1c1ddbd2</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -2521,7 +2517,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -2548,7 +2544,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>3-Yr CAGR / Shift</t>
+          <t>3-Yr Shift</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -2887,7 +2883,7 @@
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -2914,7 +2910,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>3-Yr CAGR / Shift</t>
+          <t>3-Yr Shift</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">

</xml_diff>